<commit_message>
chore: Object(Container) 상호작용 테스트 완료
# 남은 기능
- 시간 차감 로직 추가 필요
- 손에 key(tool)들고 있는경우 제대로 잠금해제 및 소모되는 key인경우 소모되는지 확인 필요
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Pool.xlsx
+++ b/JsonConverter/ExcelFiles/Pool.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>초기 생성될 수치</t>
   </si>
@@ -40,6 +40,15 @@
   </si>
   <si>
     <t>InteractableContainer_Prefab</t>
+  </si>
+  <si>
+    <t>Effect_High</t>
+  </si>
+  <si>
+    <t>Effect_Low</t>
+  </si>
+  <si>
+    <t>Effect_Normal</t>
   </si>
 </sst>
 </file>
@@ -343,9 +352,30 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="7" ht="17.25" customHeight="1"/>
-    <row r="8" ht="17.25" customHeight="1"/>
-    <row r="9" ht="17.25" customHeight="1"/>
+    <row r="7" ht="17.25" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="9" ht="17.25" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1.0</v>
+      </c>
+    </row>
     <row r="10" ht="17.25" customHeight="1"/>
     <row r="11" ht="17.25" customHeight="1"/>
     <row r="12" ht="17.25" customHeight="1"/>

</xml_diff>